<commit_message>
removed the time enum mappers to time library
</commit_message>
<xml_diff>
--- a/sheets/time_test_sheet.xlsx
+++ b/sheets/time_test_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\OdinAnalytics\sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26409539-CAA8-4966-A579-A25503D74706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880976B5-4305-4D1E-8AF1-71993B4CBFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{4F0FB8F6-FBCA-4404-B166-FFC6556ED016}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{4F0FB8F6-FBCA-4404-B166-FFC6556ED016}"/>
   </bookViews>
   <sheets>
     <sheet name="boolean_logic_dates" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="49">
   <si>
     <t>NYB</t>
   </si>
@@ -159,19 +159,28 @@
     <t>Stub_Type</t>
   </si>
   <si>
-    <t>ACT/ACT</t>
+    <t>Notional</t>
+  </si>
+  <si>
+    <t>Calc_Type</t>
+  </si>
+  <si>
+    <t>flat</t>
   </si>
   <si>
     <t>SA</t>
   </si>
   <si>
-    <t>Backwards</t>
+    <t>backwards</t>
   </si>
   <si>
-    <t>Notional</t>
+    <t>Payment_Date_Rule</t>
   </si>
   <si>
-    <t>shortlast</t>
+    <t>Act/360</t>
+  </si>
+  <si>
+    <t>LF</t>
   </si>
 </sst>
 </file>
@@ -685,25 +694,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FA05541-6074-4C5E-B131-7466FA391955}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B1:L18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B1" t="str">
         <f>ComputeDate!C2</f>
         <v>Dictionary_ComputeDate_$1$2:0</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F5" t="s">
         <v>3</v>
       </c>
@@ -726,7 +735,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F6" s="1">
         <v>44746</v>
       </c>
@@ -749,7 +758,7 @@
         <v>45074</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>0</v>
       </c>
@@ -772,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="E8" s="2" t="s">
         <v>5</v>
       </c>
@@ -805,7 +814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>1</v>
       </c>
@@ -828,7 +837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="E11" s="2" t="s">
         <v>5</v>
       </c>
@@ -861,7 +870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>4</v>
       </c>
@@ -884,7 +893,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="E14" s="2" t="s">
         <v>5</v>
       </c>
@@ -917,7 +926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="5:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:12" x14ac:dyDescent="0.3">
       <c r="F17" t="s">
         <v>6</v>
       </c>
@@ -940,7 +949,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="5:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:12" x14ac:dyDescent="0.3">
       <c r="E18" s="2" t="s">
         <v>7</v>
       </c>
@@ -982,18 +991,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFECD9EC-9790-480B-9B33-A26F15505398}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:M54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>21</v>
       </c>
@@ -1005,7 +1014,7 @@
       <c r="H2" s="13"/>
       <c r="I2" s="14"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
@@ -1025,7 +1034,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>39097</v>
       </c>
@@ -1061,7 +1070,7 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>39097</v>
       </c>
@@ -1095,7 +1104,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>39097</v>
       </c>
@@ -1129,7 +1138,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>39355</v>
       </c>
@@ -1163,7 +1172,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>39355</v>
       </c>
@@ -1197,7 +1206,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>39355</v>
       </c>
@@ -1231,7 +1240,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>39097</v>
       </c>
@@ -1265,7 +1274,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>39113</v>
       </c>
@@ -1299,7 +1308,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>39141</v>
       </c>
@@ -1333,7 +1342,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>38960</v>
       </c>
@@ -1367,7 +1376,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>39141</v>
       </c>
@@ -1401,7 +1410,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>39127</v>
       </c>
@@ -1435,7 +1444,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>39139</v>
       </c>
@@ -1469,7 +1478,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>39507</v>
       </c>
@@ -1503,7 +1512,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>39507</v>
       </c>
@@ -1537,7 +1546,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>39507</v>
       </c>
@@ -1571,7 +1580,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>39141</v>
       </c>
@@ -1605,7 +1614,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>39386</v>
       </c>
@@ -1639,7 +1648,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>39325</v>
       </c>
@@ -1673,7 +1682,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>39507</v>
       </c>
@@ -1707,7 +1716,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>39691</v>
       </c>
@@ -1741,7 +1750,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>39872</v>
       </c>
@@ -1775,7 +1784,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
         <v>20</v>
       </c>
@@ -1787,7 +1796,7 @@
       <c r="H27" s="13"/>
       <c r="I27" s="14"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>17</v>
       </c>
@@ -1807,7 +1816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>39097</v>
       </c>
@@ -1829,7 +1838,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>39097</v>
       </c>
@@ -1851,7 +1860,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>39097</v>
       </c>
@@ -1873,7 +1882,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>39355</v>
       </c>
@@ -1895,7 +1904,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>39355</v>
       </c>
@@ -1917,7 +1926,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>39355</v>
       </c>
@@ -1939,7 +1948,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>39097</v>
       </c>
@@ -1961,7 +1970,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>39113</v>
       </c>
@@ -1983,7 +1992,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>39141</v>
       </c>
@@ -2005,7 +2014,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>38960</v>
       </c>
@@ -2027,7 +2036,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>39141</v>
       </c>
@@ -2049,7 +2058,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>39127</v>
       </c>
@@ -2071,7 +2080,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>39139</v>
       </c>
@@ -2093,7 +2102,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>39507</v>
       </c>
@@ -2115,7 +2124,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>39507</v>
       </c>
@@ -2137,7 +2146,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>39507</v>
       </c>
@@ -2159,7 +2168,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>39141</v>
       </c>
@@ -2181,7 +2190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>39386</v>
       </c>
@@ -2203,7 +2212,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>39325</v>
       </c>
@@ -2225,7 +2234,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>39507</v>
       </c>
@@ -2247,7 +2256,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>39691</v>
       </c>
@@ -2269,7 +2278,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="5">
         <v>39872</v>
       </c>
@@ -2291,12 +2300,12 @@
         <v>180</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>17</v>
       </c>
@@ -2307,7 +2316,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>39097</v>
       </c>
@@ -2326,16 +2335,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08C45751-0031-44E3-951D-7C59C3883439}">
   <dimension ref="B2:K20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C2" t="str">
         <f>_xll.oxlDictionary(B3:B6,C3:C6)</f>
         <v>Dictionary_ComputeDate_$1$2:0</v>
@@ -2345,7 +2354,7 @@
         <v>Dictionary_ComputeDate_$1$10:0</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>26</v>
       </c>
@@ -2366,7 +2375,7 @@
         <v>46336</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>27</v>
       </c>
@@ -2386,7 +2395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>28</v>
       </c>
@@ -2406,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>29</v>
       </c>
@@ -2420,12 +2429,12 @@
         <v>8M</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C8" s="1">
         <f>_xll.oxlComputeDate(B3:C6)</f>
         <v>45407</v>
@@ -2435,7 +2444,7 @@
         <v>46344</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C9" s="1">
         <f>_xll.oxlComputeDate(B3:B6,C3:C6)</f>
         <v>45407</v>
@@ -2445,7 +2454,7 @@
         <v>46344</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C10" s="1">
         <f>_xll.oxlComputeDate(C2)</f>
         <v>45407</v>
@@ -2455,19 +2464,19 @@
         <v>46344</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C11" s="1">
         <f>_xll.oxlComputeDate(C3,C4,C5,C6)</f>
         <v>45407</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K12" t="str">
         <f>_xll.oxlDictionary(J13:J15,K13:K15)</f>
         <v>Dictionary_ComputeDate_$11$10:0</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
       <c r="J13" t="s">
         <v>26</v>
       </c>
@@ -2475,7 +2484,7 @@
         <v>46344</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
       <c r="J14" t="s">
         <v>33</v>
       </c>
@@ -2483,7 +2492,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="J15" t="s">
         <v>29</v>
       </c>
@@ -2491,19 +2500,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="11:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K18" s="1">
         <f>_xll.oxlAddBusinessDays(K13,K14,K15)</f>
         <v>46336</v>
       </c>
     </row>
-    <row r="19" spans="11:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K19" s="1">
         <f>_xll.oxlAddBusinessDays(J13:J15,K13:K15)</f>
         <v>46336</v>
       </c>
     </row>
-    <row r="20" spans="11:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K20" s="1">
         <f>_xll.oxlAddBusinessDays(K12)</f>
         <v>46336</v>
@@ -2516,21 +2525,29 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70F557B0-F1EA-4C34-B59A-53CDA196B303}">
-  <dimension ref="B2:V20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:T63"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>34</v>
       </c>
@@ -2538,103 +2555,95 @@
         <v>45660</v>
       </c>
       <c r="E2" t="str">
-        <f>_xll.oxlDictionary(B2:B9,C2:C9)</f>
-        <v>Dictionary_CashFlow_$1$4:11</v>
-      </c>
-      <c r="G2" s="1">
-        <f t="array" ref="G2:T20">_xll.oxlGenerateCashFlows(E2)</f>
-        <v>45598</v>
-      </c>
-      <c r="H2" s="1">
-        <v>45779</v>
-      </c>
-      <c r="I2" s="1">
-        <v>45598</v>
-      </c>
-      <c r="J2" s="1">
-        <v>45779</v>
-      </c>
-      <c r="K2" s="1">
-        <v>45598</v>
-      </c>
-      <c r="L2" s="1">
-        <v>45779</v>
-      </c>
-      <c r="M2" s="16">
-        <v>1000000</v>
-      </c>
-      <c r="N2">
-        <v>0.05</v>
-      </c>
-      <c r="O2" s="16">
-        <v>24772.063777228836</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>181</v>
-      </c>
-      <c r="R2">
-        <v>0.49544127554457673</v>
+        <f>_xll.oxlDictionary(B2:B11,C2:C11)</f>
+        <v>Dictionary_CashFlow_$1$4:2</v>
+      </c>
+      <c r="G2" s="1" t="str">
+        <f t="array" ref="G2:T63">_xll.oxlGenerateCashFlows(E2)</f>
+        <v>Unadj_Start_Date</v>
+      </c>
+      <c r="H2" s="1" t="str">
+        <v>Unadj_End_Date</v>
+      </c>
+      <c r="I2" s="1" t="str">
+        <v>Start_Date</v>
+      </c>
+      <c r="J2" s="1" t="str">
+        <v>End_Date</v>
+      </c>
+      <c r="K2" s="1" t="str">
+        <v>Fixing_Date</v>
+      </c>
+      <c r="L2" s="1" t="str">
+        <v>Payment_Date</v>
+      </c>
+      <c r="M2" s="16" t="str">
+        <v>Notional</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Rate</v>
+      </c>
+      <c r="O2" s="16" t="str">
+        <v>Fwd_Cashflow_PV</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Cashflow_NPV</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Day_Count</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Day_Count_Fraction</v>
       </c>
       <c r="S2" t="str">
-        <v>USD</v>
+        <v>Currency</v>
       </c>
       <c r="T2" t="str">
-        <v>Fixed</v>
-      </c>
-      <c r="U2">
-        <f>_xll.oxlComputeYearFraction(G2,H2,"ACT:ACT")</f>
-        <v>0.49544127554457673</v>
-      </c>
-      <c r="V2">
-        <f>U2-R2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
+        <v>Cashflow_Type</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>35</v>
       </c>
       <c r="C3" s="1">
-        <v>47605</v>
+        <v>47575</v>
       </c>
       <c r="G3" s="1">
-        <v>45779</v>
+        <v>45660</v>
       </c>
       <c r="H3" s="1">
-        <v>45963</v>
+        <v>45932</v>
       </c>
       <c r="I3" s="1">
-        <v>45779</v>
+        <v>45660</v>
       </c>
       <c r="J3" s="1">
-        <v>45963</v>
+        <v>45932</v>
       </c>
       <c r="K3" s="1">
-        <v>45779</v>
+        <v>45660</v>
       </c>
       <c r="L3" s="1">
-        <v>45963</v>
+        <v>45933</v>
       </c>
       <c r="M3" s="16">
         <v>1000000</v>
       </c>
       <c r="N3">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O3" s="16">
-        <v>25205.479452054798</v>
+        <v>7555555.555555555</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>184</v>
+        <v>272</v>
       </c>
       <c r="R3">
-        <v>0.50410958904109593</v>
+        <v>0.75555555555555554</v>
       </c>
       <c r="S3" t="str">
         <v>USD</v>
@@ -2642,57 +2651,49 @@
       <c r="T3" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U3">
-        <f>_xll.oxlComputeYearFraction(G3,H3,"ACT:ACT")</f>
-        <v>0.50410958904109593</v>
-      </c>
-      <c r="V3">
-        <f t="shared" ref="V3:V13" si="0">U3-R3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C4">
         <v>1000000</v>
       </c>
       <c r="G4" s="1">
-        <v>45963</v>
+        <v>45932</v>
       </c>
       <c r="H4" s="1">
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="I4" s="1">
-        <v>45963</v>
+        <v>45932</v>
       </c>
       <c r="J4" s="1">
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="K4" s="1">
-        <v>45963</v>
+        <v>45932</v>
       </c>
       <c r="L4" s="1">
-        <v>46144</v>
+        <v>46115</v>
       </c>
       <c r="M4" s="16">
         <v>1000000</v>
       </c>
       <c r="N4">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O4" s="16">
-        <v>24794.520547945209</v>
+        <v>5055555.555555555</v>
       </c>
       <c r="P4">
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R4">
-        <v>0.49589041095890413</v>
+        <v>0.50555555555555554</v>
       </c>
       <c r="S4" t="str">
         <v>USD</v>
@@ -2700,57 +2701,49 @@
       <c r="T4" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U4">
-        <f>_xll.oxlComputeYearFraction(G4,H4,"ACT:ACT")</f>
-        <v>0.49589041095890413</v>
-      </c>
-      <c r="V4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>36</v>
       </c>
       <c r="C5">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="G5" s="1">
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="H5" s="1">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="I5" s="1">
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="J5" s="1">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="K5" s="1">
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="L5" s="1">
-        <v>46328</v>
+        <v>46300</v>
       </c>
       <c r="M5" s="16">
         <v>1000000</v>
       </c>
       <c r="N5">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O5" s="16">
-        <v>25205.479452054798</v>
+        <v>5083333.333333333</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R5">
-        <v>0.50410958904109593</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="S5" t="str">
         <v>USD</v>
@@ -2758,57 +2751,49 @@
       <c r="T5" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U5">
-        <f>_xll.oxlComputeYearFraction(G5,H5,"ACT:ACT")</f>
-        <v>0.50410958904109593</v>
-      </c>
-      <c r="V5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="H6" s="1">
-        <v>46509</v>
+        <v>46479</v>
       </c>
       <c r="I6" s="1">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="J6" s="1">
-        <v>46509</v>
+        <v>46479</v>
       </c>
       <c r="K6" s="1">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="L6" s="1">
-        <v>46509</v>
+        <v>46482</v>
       </c>
       <c r="M6" s="16">
         <v>1000000</v>
       </c>
       <c r="N6">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O6" s="16">
-        <v>24794.520547945209</v>
+        <v>5055555.555555555</v>
       </c>
       <c r="P6">
         <v>0</v>
       </c>
       <c r="Q6">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R6">
-        <v>0.49589041095890413</v>
+        <v>0.50555555555555554</v>
       </c>
       <c r="S6" t="str">
         <v>USD</v>
@@ -2816,57 +2801,49 @@
       <c r="T6" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U6">
-        <f>_xll.oxlComputeYearFraction(G6,H6,"ACT:ACT")</f>
-        <v>0.49589041095890413</v>
-      </c>
-      <c r="V6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G7" s="1">
-        <v>46509</v>
+        <v>46479</v>
       </c>
       <c r="H7" s="1">
-        <v>46693</v>
+        <v>46662</v>
       </c>
       <c r="I7" s="1">
-        <v>46509</v>
+        <v>46479</v>
       </c>
       <c r="J7" s="1">
-        <v>46693</v>
+        <v>46662</v>
       </c>
       <c r="K7" s="1">
-        <v>46509</v>
+        <v>46479</v>
       </c>
       <c r="L7" s="1">
-        <v>46693</v>
+        <v>46664</v>
       </c>
       <c r="M7" s="16">
         <v>1000000</v>
       </c>
       <c r="N7">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O7" s="16">
-        <v>25205.479452054798</v>
+        <v>5083333.333333333</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R7">
-        <v>0.50410958904109593</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="S7" t="str">
         <v>USD</v>
@@ -2874,57 +2851,49 @@
       <c r="T7" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U7">
-        <f>_xll.oxlComputeYearFraction(G7,H7,"ACT:ACT")</f>
-        <v>0.50410958904109593</v>
-      </c>
-      <c r="V7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G8" s="1">
-        <v>46693</v>
+        <v>46662</v>
       </c>
       <c r="H8" s="1">
-        <v>46875</v>
+        <v>46845</v>
       </c>
       <c r="I8" s="1">
-        <v>46693</v>
+        <v>46662</v>
       </c>
       <c r="J8" s="1">
-        <v>46875</v>
+        <v>46845</v>
       </c>
       <c r="K8" s="1">
-        <v>46693</v>
+        <v>46662</v>
       </c>
       <c r="L8" s="1">
-        <v>46875</v>
+        <v>46846</v>
       </c>
       <c r="M8" s="16">
         <v>1000000</v>
       </c>
       <c r="N8">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O8" s="16">
-        <v>24885.84474885845</v>
+        <v>5083333.333333333</v>
       </c>
       <c r="P8">
         <v>0</v>
       </c>
       <c r="Q8">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="R8">
-        <v>0.49771689497716892</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="S8" t="str">
         <v>USD</v>
@@ -2932,57 +2901,49 @@
       <c r="T8" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U8">
-        <f>_xll.oxlComputeYearFraction(G8,H8,"ACT:ACT")</f>
-        <v>0.49771689497716892</v>
-      </c>
-      <c r="V8">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G9" s="1">
-        <v>46875</v>
+        <v>46845</v>
       </c>
       <c r="H9" s="1">
-        <v>47059</v>
+        <v>47028</v>
       </c>
       <c r="I9" s="1">
-        <v>46875</v>
+        <v>46845</v>
       </c>
       <c r="J9" s="1">
-        <v>47059</v>
+        <v>47028</v>
       </c>
       <c r="K9" s="1">
-        <v>46875</v>
+        <v>46845</v>
       </c>
       <c r="L9" s="1">
-        <v>47059</v>
+        <v>47029</v>
       </c>
       <c r="M9" s="16">
         <v>1000000</v>
       </c>
       <c r="N9">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O9" s="16">
-        <v>25136.612021857924</v>
+        <v>5083333.333333333</v>
       </c>
       <c r="P9">
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R9">
-        <v>0.50273224043715847</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="S9" t="str">
         <v>USD</v>
@@ -2990,51 +2951,49 @@
       <c r="T9" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U9">
-        <f>_xll.oxlComputeYearFraction(G9,H9,"ACT:ACT")</f>
-        <v>0.50273224043715847</v>
-      </c>
-      <c r="V9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
       <c r="G10" s="1">
-        <v>47059</v>
+        <v>47028</v>
       </c>
       <c r="H10" s="1">
-        <v>47240</v>
+        <v>47210</v>
       </c>
       <c r="I10" s="1">
-        <v>47059</v>
+        <v>47028</v>
       </c>
       <c r="J10" s="1">
-        <v>47240</v>
+        <v>47210</v>
       </c>
       <c r="K10" s="1">
-        <v>47059</v>
+        <v>47028</v>
       </c>
       <c r="L10" s="1">
-        <v>47240</v>
+        <v>47211</v>
       </c>
       <c r="M10" s="16">
         <v>1000000</v>
       </c>
       <c r="N10">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O10" s="16">
-        <v>24772.063777228836</v>
+        <v>5055555.555555555</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R10">
-        <v>0.49544127554457673</v>
+        <v>0.50555555555555554</v>
       </c>
       <c r="S10" t="str">
         <v>USD</v>
@@ -3042,51 +3001,50 @@
       <c r="T10" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U10">
-        <f>_xll.oxlComputeYearFraction(G10,H10,"ACT:ACT")</f>
-        <v>0.49544127554457673</v>
-      </c>
-      <c r="V10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="str">
+        <f>_xll.oxlDictionary(B19:B20,C19:C20)</f>
+        <v>Dictionary_CashFlow_$10$2:1</v>
+      </c>
       <c r="G11" s="1">
-        <v>47240</v>
+        <v>47210</v>
       </c>
       <c r="H11" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="I11" s="1">
-        <v>47240</v>
+        <v>47210</v>
       </c>
       <c r="J11" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="K11" s="1">
-        <v>47240</v>
+        <v>47210</v>
       </c>
       <c r="L11" s="1">
-        <v>47424</v>
+        <v>47394</v>
       </c>
       <c r="M11" s="16">
         <v>1000000</v>
       </c>
       <c r="N11">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O11" s="16">
-        <v>25205.479452054798</v>
+        <v>5083333.333333333</v>
       </c>
       <c r="P11">
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R11">
-        <v>0.50410958904109593</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="S11" t="str">
         <v>USD</v>
@@ -3094,51 +3052,43 @@
       <c r="T11" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U11">
-        <f>_xll.oxlComputeYearFraction(G11,H11,"ACT:ACT")</f>
-        <v>0.50410958904109593</v>
-      </c>
-      <c r="V11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G12" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="H12" s="1">
-        <v>47605</v>
+        <v>47575</v>
       </c>
       <c r="I12" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="J12" s="1">
-        <v>47605</v>
+        <v>47575</v>
       </c>
       <c r="K12" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="L12" s="1">
-        <v>47605</v>
+        <v>47576</v>
       </c>
       <c r="M12" s="16">
         <v>1000000</v>
       </c>
       <c r="N12">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="O12" s="16">
-        <v>24794.520547945209</v>
+        <v>5055555.555555555</v>
       </c>
       <c r="P12">
         <v>0</v>
       </c>
       <c r="Q12">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R12">
-        <v>0.49589041095890413</v>
+        <v>0.50555555555555554</v>
       </c>
       <c r="S12" t="str">
         <v>USD</v>
@@ -3146,33 +3096,25 @@
       <c r="T12" t="str">
         <v>Fixed</v>
       </c>
-      <c r="U12">
-        <f>_xll.oxlComputeYearFraction(G12,H12,"ACT:ACT")</f>
-        <v>0.49589041095890413</v>
-      </c>
-      <c r="V12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G13" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="H13" s="1">
-        <v>47605</v>
+        <v>47575</v>
       </c>
       <c r="I13" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="J13" s="1">
-        <v>47605</v>
+        <v>47575</v>
       </c>
       <c r="K13" s="1">
-        <v>47424</v>
+        <v>47393</v>
       </c>
       <c r="L13" s="1">
-        <v>47605</v>
+        <v>47576</v>
       </c>
       <c r="M13" s="16">
         <v>1000000</v>
@@ -3187,10 +3129,10 @@
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R13">
-        <v>0.49589041095890413</v>
+        <v>0.50555555555555554</v>
       </c>
       <c r="S13" t="str">
         <v>USD</v>
@@ -3198,16 +3140,8 @@
       <c r="T13" t="str">
         <v>Principal</v>
       </c>
-      <c r="U13">
-        <f>_xll.oxlComputeYearFraction(G13,H13,"ACT:ACT")</f>
-        <v>0.49589041095890413</v>
-      </c>
-      <c r="V13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G14" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3251,7 +3185,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G15" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3295,7 +3229,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G16" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3339,7 +3273,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="17" spans="7:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G17" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3383,7 +3317,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="18" spans="7:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G18" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3427,7 +3361,13 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="19" spans="7:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
       <c r="G19" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3471,7 +3411,13 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="20" spans="7:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" t="s">
+        <v>0</v>
+      </c>
       <c r="G20" s="1" t="e">
         <v>#N/A</v>
       </c>
@@ -3512,6 +3458,1898 @@
         <v>#N/A</v>
       </c>
       <c r="T20" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M21" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O21" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T21" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M22" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O22" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T22" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M23" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O23" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T23" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M24" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O24" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T24" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M25" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O25" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T25" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M26" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O26" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T26" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M27" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O27" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T27" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M28" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O28" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T28" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M29" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O29" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T29" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M30" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O30" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T30" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M31" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O31" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T31" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="G32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M32" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O32" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T32" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="33" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M33" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O33" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T33" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="34" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M34" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O34" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T34" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="35" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M35" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O35" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T35" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="36" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M36" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O36" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T36" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="37" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M37" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O37" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T37" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="38" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M38" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O38" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T38" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="39" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M39" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O39" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T39" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="40" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M40" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O40" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T40" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="41" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M41" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O41" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T41" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="42" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M42" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O42" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T42" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="43" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M43" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O43" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T43" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="44" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M44" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O44" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T44" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="45" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M45" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O45" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T45" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="46" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M46" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O46" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T46" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="47" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M47" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O47" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T47" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="48" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M48" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O48" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T48" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="49" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M49" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O49" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T49" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="50" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M50" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O50" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T50" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="51" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M51" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O51" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T51" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="52" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M52" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O52" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T52" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="53" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M53" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O53" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T53" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="54" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M54" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O54" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T54" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="55" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M55" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O55" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T55" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="56" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M56" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O56" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T56" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="57" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M57" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N57" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O57" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P57" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q57" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R57" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S57" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T57" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="58" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M58" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N58" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O58" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P58" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q58" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R58" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S58" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T58" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="59" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M59" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N59" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O59" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P59" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q59" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R59" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S59" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T59" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="60" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M60" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N60" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O60" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P60" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q60" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R60" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S60" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T60" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="61" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M61" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N61" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O61" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P61" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q61" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R61" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S61" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T61" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="62" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M62" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N62" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O62" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P62" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q62" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R62" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S62" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T62" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="63" spans="7:20" x14ac:dyDescent="0.3">
+      <c r="G63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="K63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M63" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="N63" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="O63" s="16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="P63" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="Q63" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="R63" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S63" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="T63" t="e">
         <v>#N/A</v>
       </c>
     </row>

</xml_diff>